<commit_message>
docs: document install/run/test, certs and allowlist rule; refresh CMDB
- CLAUDE.md: add an Install / run / test section (npm workspaces, Docker
  Compose, verify), a certificates note (mTLS PKI lives in ~/shieldtest-pki,
  never committed), the relationship to shieldtest-lab (telemetry feeds the WRS
  read-only), and an explicit "no out-of-allowlist load generation" rule.
- docs/cmdb (build_cmdb.py + regenerated .xlsx): Change Log entries for admin
  SSH access (dedicated key), the VPS 2 lab runner going live via the VPS 1
  SSH tunnel and handling a class-C job; Secrets Registry rows for the two SSH
  keys (registry only, no values). PENDING line reduced accordingly.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NqeUB7qvNzcfkEHmm2Z5Cd
</commit_message>
<xml_diff>
--- a/docs/cmdb/shieldtest-cmdb.xlsx
+++ b/docs/cmdb/shieldtest-cmdb.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPS Inventory" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network &amp; Firewall" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles &amp; Services" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositories &amp; CICD" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoints" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment Variables" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secrets Registry" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engagement" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="VPS Inventory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Network &amp; Firewall" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Roles &amp; Services" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Repositories &amp; CICD" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Endpoints" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Environment Variables" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Secrets Registry" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Engagement" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Change Log" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -622,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -798,13 +798,47 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr"/>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>PENDING: VPS 2 lab runner (host-lab.sh) + scrubber hook PROTECTION_METRICS_URL + full pretest-cra-l7 suite.</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr"/>
+          <t>Admin SSH access established from workstation via dedicated key ~/.ssh/shieldtest_vps (ed25519, authorized_keys on VPS1+VPS2). VPS1 /health=ok (build 184), VPS2 verified.</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Claude/abdelha</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>VPS 2 lab runner LIVE: systemd shieldtest-lab-runner active (RUNNER_ID=vm32046), repo /opt/shieldtest-lab @ c752a06. Reaches VPS1 API via SSH tunnel (ssh -L 127.0.0.1:8080 -&gt; VPS1:8080, key /root/.ssh/vps1_tunnel). Claimed+handled class-C job udp_dns_reflection -&gt; UNMITIGATED_BASELINE (bounded dns burst, 720 pkts, within caps).</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Claude/abdelha</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>PENDING: scrubber hook PROTECTION_METRICS_URL (VPS1 protection=false) + full pretest-cra-l7 suite. Reminder: rotate the 3 generated secrets (transcript-exposed).</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2636,7 +2670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2920,44 +2954,108 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
+          <t>Admin SSH key: shieldtest_vps</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>workstation -&gt; VPS1+VPS2 admin login</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>authorized_keys on both VPS</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Workstation ~/.ssh (no passphrase)</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>ssh-keygen ed25519</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>active (2026-09-09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Tunnel SSH key: vps1_tunnel</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>VPS2 -&gt; VPS1 API tunnel (ssh -L 8080)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>VPS2 /root/.ssh; authorized on VPS1</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>VPS2 filesystem</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>ssh-keygen</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
           <t>PROTECTION_METRICS_URL</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>scrubber hook endpoint</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>VPS 1 env</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Password manager / infra note</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>WEDOS scrubber</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>PENDING — not yet wired</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Reminder: the three generated secrets were pasted into a chat transcript on 2026-09-09; rotate if that transcript is considered exposed.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>After first SSH login on each VPS: change root password, install an admin SSH key, disable password auth.</t>
         </is>

</xml_diff>

<commit_message>
docs: document install/run/test, certs and allowlist rule; refresh CMDB (#10)
- CLAUDE.md: add an Install / run / test section (npm workspaces, Docker
  Compose, verify), a certificates note (mTLS PKI lives in ~/shieldtest-pki,
  never committed), the relationship to shieldtest-lab (telemetry feeds the WRS
  read-only), and an explicit "no out-of-allowlist load generation" rule.
- docs/cmdb (build_cmdb.py + regenerated .xlsx): Change Log entries for admin
  SSH access (dedicated key), the VPS 2 lab runner going live via the VPS 1
  SSH tunnel and handling a class-C job; Secrets Registry rows for the two SSH
  keys (registry only, no values). PENDING line reduced accordingly.


Claude-Session: https://claude.ai/code/session_01NqeUB7qvNzcfkEHmm2Z5Cd

Co-authored-by: ABDELHA TAYEB <abdelhatayeb@macbook-air-de-abdelha.home>
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cmdb/shieldtest-cmdb.xlsx
+++ b/docs/cmdb/shieldtest-cmdb.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPS Inventory" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network &amp; Firewall" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles &amp; Services" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositories &amp; CICD" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoints" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment Variables" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secrets Registry" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engagement" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="VPS Inventory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Network &amp; Firewall" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Roles &amp; Services" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Repositories &amp; CICD" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Endpoints" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Environment Variables" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Secrets Registry" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Engagement" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Change Log" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -622,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -798,13 +798,47 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr"/>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>PENDING: VPS 2 lab runner (host-lab.sh) + scrubber hook PROTECTION_METRICS_URL + full pretest-cra-l7 suite.</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr"/>
+          <t>Admin SSH access established from workstation via dedicated key ~/.ssh/shieldtest_vps (ed25519, authorized_keys on VPS1+VPS2). VPS1 /health=ok (build 184), VPS2 verified.</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Claude/abdelha</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>VPS 2 lab runner LIVE: systemd shieldtest-lab-runner active (RUNNER_ID=vm32046), repo /opt/shieldtest-lab @ c752a06. Reaches VPS1 API via SSH tunnel (ssh -L 127.0.0.1:8080 -&gt; VPS1:8080, key /root/.ssh/vps1_tunnel). Claimed+handled class-C job udp_dns_reflection -&gt; UNMITIGATED_BASELINE (bounded dns burst, 720 pkts, within caps).</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Claude/abdelha</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>PENDING: scrubber hook PROTECTION_METRICS_URL (VPS1 protection=false) + full pretest-cra-l7 suite. Reminder: rotate the 3 generated secrets (transcript-exposed).</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2636,7 +2670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2920,44 +2954,108 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
+          <t>Admin SSH key: shieldtest_vps</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>workstation -&gt; VPS1+VPS2 admin login</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>authorized_keys on both VPS</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Workstation ~/.ssh (no passphrase)</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>ssh-keygen ed25519</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>active (2026-09-09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Tunnel SSH key: vps1_tunnel</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>VPS2 -&gt; VPS1 API tunnel (ssh -L 8080)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>VPS2 /root/.ssh; authorized on VPS1</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>VPS2 filesystem</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>ssh-keygen</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
           <t>PROTECTION_METRICS_URL</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>scrubber hook endpoint</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>VPS 1 env</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Password manager / infra note</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>WEDOS scrubber</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>PENDING — not yet wired</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Reminder: the three generated secrets were pasted into a chat transcript on 2026-09-09; rotate if that transcript is considered exposed.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>After first SSH login on each VPS: change root password, install an admin SSH key, disable password auth.</t>
         </is>

</xml_diff>